<commit_message>
Add MoMo Quick Link button to UI
Insert a new 'MoMo Quick Link' button next to the existing custom QR button in index.html that opens https://kiehtt.vercel.app/ in a new tab. The button has a custom background color (#ae2070) and a left margin for spacing. Also includes an updated VietQR.xlsx binary file.
</commit_message>
<xml_diff>
--- a/VietQR.xlsx
+++ b/VietQR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\qr_bank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D935621E-98C6-4BF7-A249-25B26C4543F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D8C712-920B-42F7-A0C8-3778E92A4BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List_bank" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="265">
   <si>
     <t>data__id</t>
   </si>
@@ -798,28 +798,37 @@
     <t>https://cdn.vietqr.io/img/momo.png</t>
   </si>
   <si>
-    <t>TCB_446</t>
-  </si>
-  <si>
     <t>TCB -iPanDa</t>
   </si>
   <si>
     <t>MS00T09548691713297</t>
   </si>
   <si>
-    <t>VIB_064</t>
-  </si>
-  <si>
     <t>064933000</t>
   </si>
   <si>
-    <t>VIB_052</t>
-  </si>
-  <si>
     <t>052004</t>
   </si>
   <si>
     <t>Template</t>
+  </si>
+  <si>
+    <t>TCB_999</t>
+  </si>
+  <si>
+    <t>VIB_000</t>
+  </si>
+  <si>
+    <t>VIB_004</t>
+  </si>
+  <si>
+    <t>Green Cofee</t>
+  </si>
+  <si>
+    <t>MOMO_IPA_HUYNHKIET</t>
+  </si>
+  <si>
+    <t>PMC2605818000000089</t>
   </si>
 </sst>
 </file>
@@ -1248,10 +1257,10 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1286,7 +1295,7 @@
         <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C3">
         <v>44699999999</v>
@@ -1324,10 +1333,10 @@
         <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1362,10 +1371,10 @@
         <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -1396,30 +1405,41 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C6" s="1"/>
+      <c r="A6">
+        <v>65</v>
+      </c>
+      <c r="B6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="E6" t="str">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$H,5,0)),"-")</f>
-        <v>-</v>
+        <v>MoMo</v>
       </c>
       <c r="F6" t="str">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$H,3,0)),"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G6" t="str">
+        <v>momo</v>
+      </c>
+      <c r="G6">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$G,4,0)),"-")</f>
-        <v>-</v>
+        <v>971025</v>
       </c>
       <c r="H6" t="str">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$G,5,0)),"-")</f>
-        <v>-</v>
+        <v>MoMo</v>
       </c>
       <c r="I6" t="str">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$G,6,0)),"-")</f>
-        <v>-</v>
+        <v>https://cdn.vietqr.io/img/momo.png</v>
       </c>
       <c r="J6" t="str">
         <f>IFERROR((VLOOKUP(A6,'API - io'!$A:$G,7,0)),"-")</f>
-        <v>-</v>
+        <v>MoMo</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -1450,7 +1470,6 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C8" s="1"/>
       <c r="E8" t="str">
         <f>IFERROR((VLOOKUP(A8,'API - io'!$A:$H,5,0)),"-")</f>
         <v>-</v>
@@ -4107,7 +4126,7 @@
         <v>9</v>
       </c>
       <c r="H1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>